<commit_message>
Immobilien: Soll/Ist-Miete, Fristen nach § 558/§ 573c BGB, Objekt-Cashflow und Aufteiler-Projekte
Seed kalibriert (realistische Margen, Darlehensbeträge, Umsatzfenster ab
Monatsanfang), Testdaten-Excel neu erzeugt.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014t19NxD4KbH4PE1CAzRRHA
</commit_message>
<xml_diff>
--- a/docs/testdaten/testdaten_darlehensregister.xlsx
+++ b/docs/testdaten/testdaten_darlehensregister.xlsx
@@ -773,7 +773,7 @@
         <v>IM-2024-005</v>
       </c>
       <c r="G7">
-        <v>2800000</v>
+        <v>2000000</v>
       </c>
       <c r="H7" t="str">
         <v>10.05.2024</v>
@@ -832,7 +832,7 @@
         <v>IM-2025-006</v>
       </c>
       <c r="G8">
-        <v>3200000</v>
+        <v>2200000</v>
       </c>
       <c r="H8" t="str">
         <v>20.08.2025</v>

</xml_diff>